<commit_message>
implement toggle for selection criteria of date range
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -444,7 +444,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="str">
-        <v>Bhawna</v>
+        <v>bhawna</v>
       </c>
       <c r="C3" s="1" t="str">
         <v>Bhawna123</v>
@@ -453,36 +453,19 @@
         <v>+917974738833</v>
       </c>
       <c r="E3" s="1" t="str">
-        <v>2026-01-13T09:27:51.998Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="str">
-        <v>anjali</v>
-      </c>
-      <c r="C4" s="1" t="str">
-        <v>Anjali123</v>
-      </c>
-      <c r="D4" s="1" t="str">
-        <v>+917909599371</v>
-      </c>
-      <c r="E4" s="1" t="str">
-        <v>2026-01-14T05:01:11.670Z</v>
+        <v>2026-01-14T07:05:38.748Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -554,54 +537,17 @@
         <v>2026-01-12T08:02:30.563Z</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="str">
-        <v>+917974738833</v>
-      </c>
-      <c r="C3" s="1" t="str">
-        <v>abcd</v>
-      </c>
-      <c r="D3" s="1" t="str">
-        <v>abbb</v>
-      </c>
-      <c r="E3" s="1" t="str">
-        <v>teacher</v>
-      </c>
-      <c r="F3" s="1" t="str">
-        <v>housewife</v>
-      </c>
-      <c r="G3" s="1" t="str">
-        <v>2026-01-06</v>
-      </c>
-      <c r="H3" s="1" t="str">
-        <v>mca</v>
-      </c>
-      <c r="I3" s="1" t="str">
-        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768296509/profiles/d7g0taqps9zhqr4mnflh.png</v>
-      </c>
-      <c r="J3" s="1" t="str">
-        <v>2026-01-13T09:28:29.550Z</v>
-      </c>
-      <c r="K3" s="1" t="str">
-        <v>dsfasfd</v>
-      </c>
-      <c r="L3" s="1" t="str">
-        <v>2026-01-13T09:28:29.550Z</v>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -625,10 +571,42 @@
         <v>true</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>registrationOpen</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>false</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>registrationStartDate</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>2026-01-13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>registrationEndDate</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>2026-01-15</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add PDF generation functionality and related assets
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -444,7 +444,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="str">
-        <v>Bhawna</v>
+        <v>bhawna_parashar</v>
       </c>
       <c r="C3" s="1" t="str">
         <v>Bhawna123</v>
@@ -453,7 +453,7 @@
         <v>+917974738833</v>
       </c>
       <c r="E3" s="1" t="str">
-        <v>2026-01-13T09:27:51.998Z</v>
+        <v>2026-01-13T13:19:18.222Z</v>
       </c>
     </row>
   </sheetData>
@@ -545,34 +545,34 @@
         <v>+917974738833</v>
       </c>
       <c r="C3" s="1" t="str">
-        <v>abcd</v>
+        <v>abcdge</v>
       </c>
       <c r="D3" s="1" t="str">
-        <v>abbb</v>
+        <v>abchde</v>
       </c>
       <c r="E3" s="1" t="str">
-        <v>teacher</v>
+        <v>dfsdfas</v>
       </c>
       <c r="F3" s="1" t="str">
-        <v>housewife</v>
+        <v>dfesdfas</v>
       </c>
       <c r="G3" s="1" t="str">
-        <v>2026-01-06</v>
+        <v>2026-01-07</v>
       </c>
       <c r="H3" s="1" t="str">
-        <v>mca</v>
+        <v>dsytgcvv</v>
       </c>
       <c r="I3" s="1" t="str">
-        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768296509/profiles/d7g0taqps9zhqr4mnflh.png</v>
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768310382/profiles/owexnl8kmdn1titmh9v2.png</v>
       </c>
       <c r="J3" s="1" t="str">
-        <v>2026-01-13T09:28:29.550Z</v>
+        <v>2026-01-13T13:19:44.407Z</v>
       </c>
       <c r="K3" s="1" t="str">
-        <v>dsfasfd</v>
+        <v>dfsdfsadfs</v>
       </c>
       <c r="L3" s="1" t="str">
-        <v>2026-01-13T09:28:29.550Z</v>
+        <v>2026-01-13T13:19:44.407Z</v>
       </c>
     </row>
   </sheetData>
@@ -605,11 +605,10 @@
         <v>twilioEnabled</v>
       </c>
       <c r="C2" s="1" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
@@ -620,6 +619,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetData/>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
@@ -665,7 +665,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
fix validation and bugs
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -473,16 +473,33 @@
         <v>2026-01-14T09:57:06.862Z</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>saket</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>Saket123</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v>2026-01-15T04:49:35.804Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L12"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -554,10 +571,389 @@
         <v>2026-01-12T08:02:30.563Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G3" s="1" t="str">
+        <v>2025-12-08</v>
+      </c>
+      <c r="H3" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I3" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768452846/profiles/mvrbn5ly0mtsmsrjmnza.png</v>
+      </c>
+      <c r="J3" s="1" t="str">
+        <v>2026-01-15T04:54:06.266Z</v>
+      </c>
+      <c r="K3" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L3" s="1" t="str">
+        <v>2026-01-15T04:54:06.266Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <v>2026-01-06</v>
+      </c>
+      <c r="H4" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453227/profiles/btfejdrfp4hg8at4f32z.png</v>
+      </c>
+      <c r="J4" s="1" t="str">
+        <v>2026-01-15T05:00:27.708Z</v>
+      </c>
+      <c r="K4" s="1" t="str">
+        <v>kjjjlk</v>
+      </c>
+      <c r="L4" s="1" t="str">
+        <v>2026-01-15T05:00:27.708Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453835/profiles/j3wb9knej3xloe3o1k61.png</v>
+      </c>
+      <c r="J5" s="1" t="str">
+        <v>2026-01-15T05:10:36.499Z</v>
+      </c>
+      <c r="K5" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L5" s="1" t="str">
+        <v>2026-01-15T05:10:36.499Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H6" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453837/profiles/d438um5deym7v3xbeeq4.png</v>
+      </c>
+      <c r="J6" s="1" t="str">
+        <v>2026-01-15T05:10:37.520Z</v>
+      </c>
+      <c r="K6" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L6" s="1" t="str">
+        <v>2026-01-15T05:10:37.520Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H7" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I7" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453837/profiles/ggbjstsk7ag35rmbg4sj.png</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <v>2026-01-15T05:10:37.746Z</v>
+      </c>
+      <c r="K7" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L7" s="1" t="str">
+        <v>2026-01-15T05:10:37.746Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H8" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I8" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453837/profiles/vp3burkolxygjbgluw21.png</v>
+      </c>
+      <c r="J8" s="1" t="str">
+        <v>2026-01-15T05:10:38.517Z</v>
+      </c>
+      <c r="K8" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L8" s="1" t="str">
+        <v>2026-01-15T05:10:38.517Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F9" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H9" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I9" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453838/profiles/cvz4rpiryaezixesz70e.png</v>
+      </c>
+      <c r="J9" s="1" t="str">
+        <v>2026-01-15T05:10:38.574Z</v>
+      </c>
+      <c r="K9" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L9" s="1" t="str">
+        <v>2026-01-15T05:10:38.574Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F10" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H10" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I10" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453838/profiles/rmafvlxtpjv5bzeoga0p.png</v>
+      </c>
+      <c r="J10" s="1" t="str">
+        <v>2026-01-15T05:10:38.664Z</v>
+      </c>
+      <c r="K10" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L10" s="1" t="str">
+        <v>2026-01-15T05:10:38.664Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H11" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I11" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453838/profiles/bhup3nd7sefeb5iuycqy.png</v>
+      </c>
+      <c r="J11" s="1" t="str">
+        <v>2026-01-15T05:10:38.704Z</v>
+      </c>
+      <c r="K11" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L11" s="1" t="str">
+        <v>2026-01-15T05:10:38.704Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <v>+910987654321</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <v>kamal</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E12" s="1" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="F12" s="1" t="str">
+        <v>housewife</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <v>2025-12-18</v>
+      </c>
+      <c r="H12" s="1" t="str">
+        <v>mca</v>
+      </c>
+      <c r="I12" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768453838/profiles/t5gaitqkhlrxwcuceeia.png</v>
+      </c>
+      <c r="J12" s="1" t="str">
+        <v>2026-01-15T05:10:38.804Z</v>
+      </c>
+      <c r="K12" s="1" t="str">
+        <v>fdfsa</v>
+      </c>
+      <c r="L12" s="1" t="str">
+        <v>2026-01-15T05:10:38.804Z</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -596,7 +992,7 @@
         <v>registrationOpen</v>
       </c>
       <c r="C3" s="1" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
     </row>
     <row r="4">
@@ -618,7 +1014,7 @@
         <v>registrationEndDate</v>
       </c>
       <c r="C5" s="1" t="str">
-        <v>2026-01-15</v>
+        <v>2026-01-16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed bug fetch username, image cropper implement and all fixed in ui section
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -490,9 +490,43 @@
         <v>2026-01-15T04:49:35.804Z</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>ashish</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>Ashish123</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>+918770924432</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v>2026-01-15T04:49:35.804Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>something new</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>Saket123</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>+917898005141</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>2026-01-16T10:12:47.851Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -952,6 +986,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:L12"/>
   </ignoredErrors>
@@ -1018,6 +1053,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
@@ -1028,6 +1064,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetData/>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
image preview and admin panel bug fix
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -456,16 +456,33 @@
         <v>2026-01-13T13:19:18.222Z</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>tester</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>Tester123</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>+918959467317</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v>2026-01-19T06:11:02.489Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -504,6 +521,9 @@
       <c r="L1" s="1" t="str">
         <v>createdAt</v>
       </c>
+      <c r="M1" s="1" t="str">
+        <v>fullName</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
@@ -575,16 +595,57 @@
         <v>2026-01-13T13:19:44.407Z</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>+918959467317</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>abcd</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>meena</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v>tttt</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>tttt</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <v>2026-01-06</v>
+      </c>
+      <c r="H4" s="1" t="str">
+        <v>dddd</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <v>https://res.cloudinary.com/ddfp1evfo/image/upload/v1768803690/profiles/jugdsuglrvavphuozycf.jpg</v>
+      </c>
+      <c r="J4" s="1" t="str">
+        <v>2026-01-19T06:21:31.271Z</v>
+      </c>
+      <c r="K4" s="1" t="str">
+        <v>ffff</v>
+      </c>
+      <c r="L4" s="1" t="str">
+        <v>2026-01-19T06:18:58.203Z</v>
+      </c>
+      <c r="M4" s="1" t="str">
+        <v>tester</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -608,9 +669,42 @@
         <v>false</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>registrationOpen</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>registrationStartDate</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>2026-01-19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>registrationEndDate</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>2026-01-23</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>